<commit_message>
update after test run: trainer argument tokenizer -> processing_class
</commit_message>
<xml_diff>
--- a/data/auxiliary/fragile_states.xlsx
+++ b/data/auxiliary/fragile_states.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\auxiliary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E96A97FB-2397-44E5-B8D8-51A026801F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2464C914-2DF2-4997-A9ED-5520D58ACB34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1453,13 +1453,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q172"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:R172"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -1511,8 +1511,11 @@
       <c r="Q1" s="1">
         <v>2023</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R1" s="1">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1564,8 +1567,11 @@
       <c r="Q2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1573,7 +1579,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1581,7 +1587,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1601,7 +1607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -1609,7 +1615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1617,7 +1623,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1628,7 +1634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1639,7 +1645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -1647,7 +1653,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -1655,7 +1661,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1663,7 +1669,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -1671,7 +1677,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -1679,7 +1685,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -1687,7 +1693,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1695,7 +1701,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>44</v>
       </c>
@@ -1703,7 +1709,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -1711,7 +1717,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -1740,7 +1746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>50</v>
       </c>
@@ -1748,7 +1754,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -1756,7 +1762,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -1764,7 +1770,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>56</v>
       </c>
@@ -1772,7 +1778,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>58</v>
       </c>
@@ -1794,8 +1800,11 @@
       <c r="Q24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -1847,8 +1856,11 @@
       <c r="Q25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>62</v>
       </c>
@@ -1856,7 +1868,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -1881,8 +1893,11 @@
       <c r="Q27">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>66</v>
       </c>
@@ -1890,7 +1905,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>68</v>
       </c>
@@ -1942,8 +1957,11 @@
       <c r="Q29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>70</v>
       </c>
@@ -1992,8 +2010,11 @@
       <c r="Q30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -2001,7 +2022,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>74</v>
       </c>
@@ -2009,7 +2030,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -2017,7 +2038,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -2066,8 +2087,11 @@
       <c r="Q34">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>80</v>
       </c>
@@ -2119,8 +2143,11 @@
       <c r="Q35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>81</v>
       </c>
@@ -2163,8 +2190,11 @@
       <c r="Q36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>83</v>
       </c>
@@ -2172,7 +2202,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>85</v>
       </c>
@@ -2180,7 +2210,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>87</v>
       </c>
@@ -2218,7 +2248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>89</v>
       </c>
@@ -2226,7 +2256,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>91</v>
       </c>
@@ -2234,7 +2264,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>93</v>
       </c>
@@ -2242,7 +2272,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>95</v>
       </c>
@@ -2262,7 +2292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>97</v>
       </c>
@@ -2270,7 +2300,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>99</v>
       </c>
@@ -2278,7 +2308,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>101</v>
       </c>
@@ -2286,7 +2316,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>103</v>
       </c>
@@ -2294,7 +2324,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>105</v>
       </c>
@@ -2302,7 +2332,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>107</v>
       </c>
@@ -2310,7 +2340,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>109</v>
       </c>
@@ -2362,8 +2392,11 @@
       <c r="Q50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>111</v>
       </c>
@@ -2379,8 +2412,11 @@
       <c r="Q51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>113</v>
       </c>
@@ -2388,7 +2424,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>115</v>
       </c>
@@ -2396,7 +2432,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>117</v>
       </c>
@@ -2404,7 +2440,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>119</v>
       </c>
@@ -2433,7 +2469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -2450,7 +2486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>123</v>
       </c>
@@ -2458,7 +2494,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>125</v>
       </c>
@@ -2466,7 +2502,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>127</v>
       </c>
@@ -2474,7 +2510,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>129</v>
       </c>
@@ -2482,7 +2518,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>131</v>
       </c>
@@ -2502,7 +2538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>133</v>
       </c>
@@ -2554,8 +2590,11 @@
       <c r="Q62">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>135</v>
       </c>
@@ -2563,7 +2602,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>137</v>
       </c>
@@ -2615,8 +2654,11 @@
       <c r="Q64">
         <v>1</v>
       </c>
-    </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>139</v>
       </c>
@@ -2624,7 +2666,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>141</v>
       </c>
@@ -2632,7 +2674,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>143</v>
       </c>
@@ -2640,7 +2682,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>145</v>
       </c>
@@ -2648,7 +2690,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>147</v>
       </c>
@@ -2656,7 +2698,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>149</v>
       </c>
@@ -2705,8 +2747,11 @@
       <c r="Q70">
         <v>1</v>
       </c>
-    </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>151</v>
       </c>
@@ -2714,7 +2759,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>153</v>
       </c>
@@ -2722,7 +2767,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>155</v>
       </c>
@@ -2730,7 +2775,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>157</v>
       </c>
@@ -2738,7 +2783,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>159</v>
       </c>
@@ -2787,8 +2832,11 @@
       <c r="Q75">
         <v>1</v>
       </c>
-    </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>161</v>
       </c>
@@ -2796,7 +2844,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>163</v>
       </c>
@@ -2804,7 +2852,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>165</v>
       </c>
@@ -2856,8 +2904,11 @@
       <c r="Q78">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>167</v>
       </c>
@@ -2865,7 +2916,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>169</v>
       </c>
@@ -2873,7 +2924,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>171</v>
       </c>
@@ -2884,7 +2935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>173</v>
       </c>
@@ -2918,8 +2969,11 @@
       <c r="Q82">
         <v>1</v>
       </c>
-    </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>175</v>
       </c>
@@ -2927,7 +2981,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>177</v>
       </c>
@@ -2974,7 +3028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>179</v>
       </c>
@@ -3017,8 +3071,11 @@
       <c r="Q85">
         <v>1</v>
       </c>
-    </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>181</v>
       </c>
@@ -3026,7 +3083,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>183</v>
       </c>
@@ -3049,7 +3106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>185</v>
       </c>
@@ -3063,7 +3120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>187</v>
       </c>
@@ -3071,7 +3128,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>189</v>
       </c>
@@ -3079,7 +3136,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>191</v>
       </c>
@@ -3122,8 +3179,11 @@
       <c r="Q91">
         <v>1</v>
       </c>
-    </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>193</v>
       </c>
@@ -3131,7 +3191,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>195</v>
       </c>
@@ -3177,8 +3237,11 @@
       <c r="Q93">
         <v>1</v>
       </c>
-    </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>197</v>
       </c>
@@ -3186,7 +3249,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>199</v>
       </c>
@@ -3194,7 +3257,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>201</v>
       </c>
@@ -3202,7 +3265,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>203</v>
       </c>
@@ -3248,8 +3311,11 @@
       <c r="Q97">
         <v>1</v>
       </c>
-    </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R97">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>205</v>
       </c>
@@ -3257,7 +3323,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>207</v>
       </c>
@@ -3265,7 +3331,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>209</v>
       </c>
@@ -3273,7 +3339,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>211</v>
       </c>
@@ -3281,7 +3347,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>213</v>
       </c>
@@ -3289,7 +3355,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>215</v>
       </c>
@@ -3317,8 +3383,11 @@
       <c r="Q103">
         <v>1</v>
       </c>
-    </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R103">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>217</v>
       </c>
@@ -3370,8 +3439,11 @@
       <c r="Q104">
         <v>1</v>
       </c>
-    </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R104">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>219</v>
       </c>
@@ -3379,7 +3451,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>221</v>
       </c>
@@ -3387,7 +3459,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>223</v>
       </c>
@@ -3410,7 +3482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>225</v>
       </c>
@@ -3418,7 +3490,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>227</v>
       </c>
@@ -3426,7 +3498,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>229</v>
       </c>
@@ -3448,8 +3520,11 @@
       <c r="Q110">
         <v>1</v>
       </c>
-    </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R110">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>231</v>
       </c>
@@ -3471,8 +3546,11 @@
       <c r="Q111">
         <v>1</v>
       </c>
-    </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R111">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>233</v>
       </c>
@@ -3480,7 +3558,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>235</v>
       </c>
@@ -3488,7 +3566,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>237</v>
       </c>
@@ -3496,7 +3574,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>239</v>
       </c>
@@ -3504,7 +3582,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>241</v>
       </c>
@@ -3512,7 +3590,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>243</v>
       </c>
@@ -3546,8 +3624,11 @@
       <c r="Q117">
         <v>1</v>
       </c>
-    </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R117">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>245</v>
       </c>
@@ -3555,7 +3636,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>247</v>
       </c>
@@ -3563,7 +3644,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>249</v>
       </c>
@@ -3571,7 +3652,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>251</v>
       </c>
@@ -3579,7 +3660,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>253</v>
       </c>
@@ -3587,7 +3668,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>255</v>
       </c>
@@ -3595,7 +3676,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>257</v>
       </c>
@@ -3603,7 +3684,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>259</v>
       </c>
@@ -3611,7 +3692,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>261</v>
       </c>
@@ -3619,7 +3700,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>263</v>
       </c>
@@ -3635,8 +3716,11 @@
       <c r="Q127">
         <v>1</v>
       </c>
-    </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R127">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>265</v>
       </c>
@@ -3644,7 +3728,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>267</v>
       </c>
@@ -3652,7 +3736,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>269</v>
       </c>
@@ -3660,7 +3744,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>271</v>
       </c>
@@ -3668,7 +3752,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>273</v>
       </c>
@@ -3703,7 +3787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>275</v>
       </c>
@@ -3711,7 +3795,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>277</v>
       </c>
@@ -3763,8 +3847,11 @@
       <c r="Q134">
         <v>1</v>
       </c>
-    </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R134">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>279</v>
       </c>
@@ -3816,8 +3903,11 @@
       <c r="Q135">
         <v>1</v>
       </c>
-    </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R135">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>281</v>
       </c>
@@ -3825,7 +3915,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>283</v>
       </c>
@@ -3868,8 +3958,11 @@
       <c r="Q137">
         <v>1</v>
       </c>
-    </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R137">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>285</v>
       </c>
@@ -3877,7 +3970,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>287</v>
       </c>
@@ -3885,7 +3978,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>289</v>
       </c>
@@ -3893,7 +3986,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>291</v>
       </c>
@@ -3901,7 +3994,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>293</v>
       </c>
@@ -3909,7 +4002,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>295</v>
       </c>
@@ -3961,8 +4054,11 @@
       <c r="Q143">
         <v>1</v>
       </c>
-    </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R143">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>297</v>
       </c>
@@ -3970,7 +4066,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>299</v>
       </c>
@@ -3978,7 +4074,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>301</v>
       </c>
@@ -4021,8 +4117,11 @@
       <c r="Q146">
         <v>1</v>
       </c>
-    </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R146">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>303</v>
       </c>
@@ -4036,7 +4135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>305</v>
       </c>
@@ -4044,7 +4143,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>307</v>
       </c>
@@ -4052,7 +4151,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>309</v>
       </c>
@@ -4098,8 +4197,11 @@
       <c r="Q150">
         <v>1</v>
       </c>
-    </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R150">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>311</v>
       </c>
@@ -4137,7 +4239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>313</v>
       </c>
@@ -4148,7 +4250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>315</v>
       </c>
@@ -4156,7 +4258,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>317</v>
       </c>
@@ -4164,7 +4266,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>319</v>
       </c>
@@ -4172,7 +4274,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>321</v>
       </c>
@@ -4180,7 +4282,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>323</v>
       </c>
@@ -4188,7 +4290,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>325</v>
       </c>
@@ -4196,7 +4298,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>327</v>
       </c>
@@ -4239,8 +4341,11 @@
       <c r="Q159">
         <v>1</v>
       </c>
-    </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R159">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>329</v>
       </c>
@@ -4248,7 +4353,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>331</v>
       </c>
@@ -4261,8 +4366,11 @@
       <c r="Q161">
         <v>1</v>
       </c>
-    </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R161">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>333</v>
       </c>
@@ -4270,7 +4378,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>335</v>
       </c>
@@ -4278,7 +4386,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>337</v>
       </c>
@@ -4286,7 +4394,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>339</v>
       </c>
@@ -4294,7 +4402,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>341</v>
       </c>
@@ -4313,8 +4421,11 @@
       <c r="Q166">
         <v>1</v>
       </c>
-    </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R166">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>343</v>
       </c>
@@ -4322,7 +4433,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>345</v>
       </c>
@@ -4330,7 +4441,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>347</v>
       </c>
@@ -4377,7 +4488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>349</v>
       </c>
@@ -4429,8 +4540,11 @@
       <c r="Q170">
         <v>1</v>
       </c>
-    </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.45">
+      <c r="R170">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>351</v>
       </c>
@@ -4438,7 +4552,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>353</v>
       </c>
@@ -4488,6 +4602,9 @@
         <v>1</v>
       </c>
       <c r="Q172">
+        <v>1</v>
+      </c>
+      <c r="R172">
         <v>1</v>
       </c>
     </row>

</xml_diff>